<commit_message>
Add staffing plan (Stellenplan) with salary assumptions
Neues Blatt Stellenplan (20 VZÄ, Gehälter, Zuschläge, DG-Anteil) speist die
Personalkosten im Rechenmodell; Konzept um Abschnitt Personal ergänzt und
Kennzahlen aktualisiert.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LU39VnhhdZH89hhaiW5MDJ
</commit_message>
<xml_diff>
--- a/seesauna-attersee/Rechenmodell_Seesauna_Attersee.xlsx
+++ b/seesauna-attersee/Rechenmodell_Seesauna_Attersee.xlsx
@@ -14,8 +14,9 @@
     <sheet name="Investition" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Umsatz" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Betriebskosten" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="GuV_10J" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Gemeinden" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Stellenplan" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="GuV_10J" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Gemeinden" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="443">
   <si>
     <t xml:space="preserve">Szenarienvergleich – Normaljahr</t>
   </si>
@@ -338,7 +339,7 @@
     <t xml:space="preserve">VZÄ</t>
   </si>
   <si>
-    <t xml:space="preserve">Kassa 4, Saunameister:innen 5, Reinigung 4, Gastro 5, Leitung/Technik 2</t>
+    <t xml:space="preserve">Basis = Blatt Stellenplan; pessimistisch +1 VZÄ</t>
   </si>
   <si>
     <t xml:space="preserve">k_fte</t>
@@ -347,7 +348,7 @@
     <t xml:space="preserve">Personalkosten je VZÄ (inkl. Lohnnebenkosten)</t>
   </si>
   <si>
-    <t xml:space="preserve">Annahme KV Freizeitbetriebe/Gastro OÖ inkl. LNK</t>
+    <t xml:space="preserve">Ø lt. Blatt Stellenplan (inkl. Zuschläge, Dienstgeberanteil, Aushilfen)</t>
   </si>
   <si>
     <t xml:space="preserve">energie</t>
@@ -999,6 +1000,198 @@
   </si>
   <si>
     <t xml:space="preserve">Break-even in % der geplanten Besuche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stellenbesetzungsplan Betreiber (Normaljahr, Gehälter = Annahmen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gehälter orientiert am KV Hotel- und Gastgewerbe (Arbeiter/Angestellte) mit marktüblicher Überzahlung im Salzkammergut – vor Verwendung mit dem aktuell gültigen KV abgleichen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Öffnungsstunden pro Tag (10–22 Uhr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vor-/Nachbereitung pro Tag (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aufheizen, Reinigung, Kassenabschluss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebstage pro Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aus Annahmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsstunden pro Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wochenarbeitszeit (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KV Hotel- und Gastgewerbe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urlaub (Wochen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urlaubsgesetz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feiertage (Tage)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gesetzliche Feiertage AT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Krankenstand (Tage, Ø)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Netto-Jahresstunden je VZÄ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verfügbare Arbeitszeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VZÄ je durchgehend besetzter Position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faustregel: 1 Dauerposition ≈ 2,7 VZÄ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gehälter pro Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inkl. Urlaubs- und Weihnachtsgeld</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zuschläge Sonn-/Feiertag, Abend (in % der Bruttogehälter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7-Tage-Betrieb; Annahme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dienstgeberanteil (SV, DB, DZ, KommSt, MVK)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Richtwert AT ca. 28–30 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aushilfen / Geringfügige (pauschal, inkl. Abgaben)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spitzen: Wochenende, Events, Sommer-Kiosk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funktion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brutto/Monat (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jahresbrutto (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zuschläge (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DG-Anteil (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personalkosten (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø Besetzung je Betriebsstunde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aufgaben / Einstufung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsleitung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leitung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesamtverantwortung, Personal, Budget, Marketing; Tagdienst + Rufbereitschaft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stv. Leitung / Gästeservice-Leitung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dienstplanung, Kassa/Rezeption, Hotelkooperationen, Events</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Haustechnik / Bademeister:in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wärmepumpe, Wasseraufbereitung, Saunaöfen, Holzofen; Bäderhygiene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saunameister:in – Teamleitung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sauna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aufgussplan, Event-Aufgüsse, Einschulung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saunameister:innen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aufgüsse, Aufsicht Saunabereich &amp; Steg, Erste Hilfe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezeption / Kassa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gästeservice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-in, Verkauf, Gutscheine, Telefon/Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reinigung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laufende Reinigung Nass-/Ruhebereiche, Wäschelogistik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koch / Köchin (Regenerierküche)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service / Theke Bistro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theke, Bademantel-Bistro, im Sommer Kiosk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe Stammpersonal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aushilfen / Geringfügige</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSONALKOSTEN GESAMT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø Personalkosten je VZÄ (→ Annahmen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personalkosten in % vom Umsatz (aktives Szenario)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lesart Spalte I: Wie viele Personen dieser Funktion im Schnitt je Betriebsstunde im Haus sind. Summe ≈ 7–8 Personen gleichzeitig; Leitung/Technik arbeiten überwiegend im Tagdienst.</t>
   </si>
   <si>
     <t xml:space="preserve">Betreiber-GuV &amp; Pachtfluss – 10 Jahre (aktives Szenario, nominal)</t>
@@ -1170,14 +1363,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="#,##0.00;\(#,##0.00\);\-"/>
     <numFmt numFmtId="167" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="168" formatCode="0.0&quot; J.&quot;"/>
     <numFmt numFmtId="169" formatCode="0"/>
-    <numFmt numFmtId="170" formatCode="@"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="@"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -1334,7 +1528,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1431,6 +1625,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1467,7 +1669,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1854,15 +2072,15 @@
       </c>
       <c r="C8" s="4" t="n">
         <f aca="false">Betriebskosten!C13</f>
-        <v>1723301.75355906</v>
+        <v>1662815.55855906</v>
       </c>
       <c r="D8" s="4" t="n">
         <f aca="false">Betriebskosten!D13</f>
-        <v>1752636.11102732</v>
+        <v>1695030.21102732</v>
       </c>
       <c r="E8" s="4" t="n">
         <f aca="false">Betriebskosten!E13</f>
-        <v>1859371.49220854</v>
+        <v>1801765.59220854</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1894,15 +2112,15 @@
       </c>
       <c r="C10" s="4" t="n">
         <f aca="false">Betriebskosten!C16</f>
-        <v>-558127.600038476</v>
+        <v>-497641.405038476</v>
       </c>
       <c r="D10" s="4" t="n">
         <f aca="false">Betriebskosten!D16</f>
-        <v>-11489.2282262407</v>
+        <v>46116.6717737592</v>
       </c>
       <c r="E10" s="4" t="n">
         <f aca="false">Betriebskosten!E16</f>
-        <v>474759.803963063</v>
+        <v>532365.703963063</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1914,15 +2132,15 @@
       </c>
       <c r="C11" s="6" t="n">
         <f aca="false">Betriebskosten!C18</f>
-        <v>-0.424375432367209</v>
+        <v>-0.378384416775787</v>
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">Betriebskosten!D18</f>
-        <v>-0.00593878983201096</v>
+        <v>0.0238377387952543</v>
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">Betriebskosten!E18</f>
-        <v>0.183059035396843</v>
+        <v>0.205270857878738</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1934,15 +2152,15 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">Betriebskosten!C24</f>
-        <v>57649.426244079</v>
+        <v>55222.8469556743</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">Betriebskosten!D24</f>
-        <v>47525.9752987974</v>
+        <v>45490.4536776339</v>
       </c>
       <c r="E12" s="4" t="n">
         <f aca="false">Betriebskosten!E24</f>
-        <v>42122.2181054755</v>
+        <v>40290.9061930512</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1954,15 +2172,15 @@
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">Betriebskosten!C25</f>
-        <v>1.60137295122442</v>
+        <v>1.53396797099095</v>
       </c>
       <c r="D13" s="6" t="n">
         <f aca="false">Betriebskosten!D25</f>
-        <v>1.00861577459248</v>
+        <v>0.965417098421772</v>
       </c>
       <c r="E13" s="6" t="n">
         <f aca="false">Betriebskosten!E25</f>
-        <v>0.736209352538242</v>
+        <v>0.704201803601349</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2038,11 +2256,11 @@
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">MAX(0,Betriebskosten!D14/Umsatz!D16-Annahmen!$D$43)</f>
-        <v>0.014061210167989</v>
+        <v>0.0438377387952543</v>
       </c>
       <c r="E17" s="9" t="n">
         <f aca="false">MAX(0,Betriebskosten!E14/Umsatz!E16-Annahmen!$E$43)</f>
-        <v>0.203059035396843</v>
+        <v>0.225270857878738</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2058,11 +2276,11 @@
       </c>
       <c r="D18" s="4" t="n">
         <f aca="false">D17*Umsatz!D16</f>
-        <v>27202.9247248944</v>
+        <v>84808.8247248943</v>
       </c>
       <c r="E18" s="4" t="n">
         <f aca="false">E17*Umsatz!E16</f>
-        <v>526629.388322432</v>
+        <v>584235.288322432</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2776,10 +2994,12 @@
       <c r="B32" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C32" s="19" t="n">
+      <c r="C32" s="24" t="n">
+        <f aca="false">D32+1</f>
         <v>21</v>
       </c>
-      <c r="D32" s="19" t="n">
+      <c r="D32" s="25" t="n">
+        <f aca="false">Stellenplan!C29</f>
         <v>20</v>
       </c>
       <c r="E32" s="19" t="n">
@@ -2805,18 +3025,19 @@
       </c>
       <c r="C33" s="7" t="n">
         <f aca="false">D33</f>
-        <v>52000</v>
-      </c>
-      <c r="D33" s="16" t="n">
-        <v>52000</v>
+        <v>49119.705</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <f aca="false">Stellenplan!H32</f>
+        <v>49119.705</v>
       </c>
       <c r="E33" s="7" t="n">
         <f aca="false">D33</f>
-        <v>52000</v>
+        <v>49119.705</v>
       </c>
       <c r="F33" s="17" t="n">
         <f aca="false">INDEX(C33:E33,1,$C$4)</f>
-        <v>52000</v>
+        <v>49119.705</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>78</v>
@@ -2888,14 +3109,14 @@
       <c r="B36" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="24" t="n">
+      <c r="C36" s="26" t="n">
         <f aca="false">D36</f>
         <v>2.2</v>
       </c>
-      <c r="D36" s="25" t="n">
+      <c r="D36" s="27" t="n">
         <v>2.2</v>
       </c>
-      <c r="E36" s="24" t="n">
+      <c r="E36" s="26" t="n">
         <f aca="false">D36</f>
         <v>2.2</v>
       </c>
@@ -3009,14 +3230,14 @@
       <c r="B41" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C41" s="26" t="n">
+      <c r="C41" s="28" t="n">
         <f aca="false">D41</f>
         <v>0.1</v>
       </c>
-      <c r="D41" s="27" t="n">
+      <c r="D41" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="E41" s="26" t="n">
+      <c r="E41" s="28" t="n">
         <f aca="false">D41</f>
         <v>0.1</v>
       </c>
@@ -3222,18 +3443,18 @@
       <c r="B50" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C50" s="28" t="n">
+      <c r="C50" s="30" t="n">
         <f aca="false">D50</f>
         <v>2029</v>
       </c>
-      <c r="D50" s="29" t="n">
+      <c r="D50" s="31" t="n">
         <v>2029</v>
       </c>
-      <c r="E50" s="28" t="n">
+      <c r="E50" s="30" t="n">
         <f aca="false">D50</f>
         <v>2029</v>
       </c>
-      <c r="F50" s="30" t="n">
+      <c r="F50" s="32" t="n">
         <f aca="false">INDEX(C50:E50,1,$C$4)</f>
         <v>2029</v>
       </c>
@@ -3608,7 +3829,7 @@
       <c r="A20" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="B20" s="31" t="n">
+      <c r="B20" s="33" t="n">
         <f aca="false">SUM(B4:B19)</f>
         <v>1427</v>
       </c>
@@ -3617,7 +3838,7 @@
       <c r="A21" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="B21" s="25" t="n">
+      <c r="B21" s="27" t="n">
         <v>1.18</v>
       </c>
       <c r="D21" s="18" t="s">
@@ -3628,7 +3849,7 @@
       <c r="A22" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="B22" s="31" t="n">
+      <c r="B22" s="33" t="n">
         <f aca="false">ROUND(B20*B21,-1)</f>
         <v>1680</v>
       </c>
@@ -3759,7 +3980,7 @@
       <c r="B7" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="F7" s="31" t="n">
+      <c r="F7" s="33" t="n">
         <f aca="false">SUM(F5:F6)</f>
         <v>300000</v>
       </c>
@@ -3803,7 +4024,7 @@
       <c r="B11" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="F11" s="31" t="n">
+      <c r="F11" s="33" t="n">
         <f aca="false">SUM(F10:F10)</f>
         <v>1848000</v>
       </c>
@@ -3910,7 +4131,7 @@
       <c r="B18" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="F18" s="31" t="n">
+      <c r="F18" s="33" t="n">
         <f aca="false">SUM(F14:F17)</f>
         <v>2247000</v>
       </c>
@@ -4076,7 +4297,7 @@
       <c r="B28" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="F28" s="31" t="n">
+      <c r="F28" s="33" t="n">
         <f aca="false">SUM(F21:F27)</f>
         <v>2768000</v>
       </c>
@@ -4180,7 +4401,7 @@
       <c r="B35" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="F35" s="31" t="n">
+      <c r="F35" s="33" t="n">
         <f aca="false">SUM(F31:F34)</f>
         <v>697000</v>
       </c>
@@ -4244,7 +4465,7 @@
       <c r="B40" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="F40" s="31" t="n">
+      <c r="F40" s="33" t="n">
         <f aca="false">SUM(F38:F39)</f>
         <v>550000</v>
       </c>
@@ -4257,7 +4478,7 @@
       <c r="B42" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="F42" s="31" t="n">
+      <c r="F42" s="33" t="n">
         <f aca="false">F7+F11+F18+F28+F35+F40</f>
         <v>8410000</v>
       </c>
@@ -4306,7 +4527,7 @@
       <c r="B45" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="E45" s="27" t="n">
+      <c r="E45" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F45" s="7" t="n">
@@ -4321,7 +4542,7 @@
       <c r="B46" s="12" t="s">
         <v>274</v>
       </c>
-      <c r="F46" s="32" t="n">
+      <c r="F46" s="34" t="n">
         <f aca="false">F42+F43+F44+F45</f>
         <v>11114656</v>
       </c>
@@ -4395,7 +4616,7 @@
       <c r="B54" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="E54" s="27" t="n">
+      <c r="E54" s="29" t="n">
         <v>0.2</v>
       </c>
       <c r="F54" s="7" t="n">
@@ -4421,7 +4642,7 @@
       <c r="B56" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="F56" s="31" t="n">
+      <c r="F56" s="33" t="n">
         <f aca="false">SUM(F53:F55)</f>
         <v>2557431.2</v>
       </c>
@@ -4434,7 +4655,7 @@
       <c r="B58" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="F58" s="32" t="n">
+      <c r="F58" s="34" t="n">
         <f aca="false">F46-F56</f>
         <v>8557224.8</v>
       </c>
@@ -4554,19 +4775,19 @@
       <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="31" t="n">
+      <c r="C6" s="33" t="n">
         <f aca="false">C4+C5</f>
         <v>36000</v>
       </c>
-      <c r="D6" s="31" t="n">
+      <c r="D6" s="33" t="n">
         <f aca="false">D4+D5</f>
         <v>47120</v>
       </c>
-      <c r="E6" s="31" t="n">
+      <c r="E6" s="33" t="n">
         <f aca="false">E4+E5</f>
         <v>57215</v>
       </c>
-      <c r="F6" s="31" t="n">
+      <c r="F6" s="33" t="n">
         <f aca="false">INDEX(C6:E6,1,Annahmen!$C$4)</f>
         <v>47120</v>
       </c>
@@ -4602,19 +4823,19 @@
       <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="26" t="n">
         <f aca="false">(Annahmen!$C$16*Annahmen!$C$14+(1-Annahmen!$C$16)*Annahmen!$C$15)*(1-Annahmen!$C$17)</f>
         <v>25.6275</v>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="26" t="n">
         <f aca="false">(Annahmen!$D$16*Annahmen!$D$14+(1-Annahmen!$D$16)*Annahmen!$D$15)*(1-Annahmen!$D$17)</f>
         <v>28.776</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="26" t="n">
         <f aca="false">(Annahmen!$E$16*Annahmen!$E$14+(1-Annahmen!$E$16)*Annahmen!$E$15)*(1-Annahmen!$E$17)</f>
         <v>31.725</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="26" t="n">
         <f aca="false">INDEX(C8:E8,1,Annahmen!$C$4)</f>
         <v>28.776</v>
       </c>
@@ -4626,19 +4847,19 @@
       <c r="B9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="26" t="n">
         <f aca="false">C8/(1+Annahmen!$C$18)</f>
         <v>22.679203539823</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="26" t="n">
         <f aca="false">D8/(1+Annahmen!$D$18)</f>
         <v>25.4654867256637</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="26" t="n">
         <f aca="false">E8/(1+Annahmen!$E$18)</f>
         <v>28.0752212389381</v>
       </c>
-      <c r="F9" s="24" t="n">
+      <c r="F9" s="26" t="n">
         <f aca="false">INDEX(C9:E9,1,Annahmen!$C$4)</f>
         <v>25.4654867256637</v>
       </c>
@@ -4770,19 +4991,19 @@
       <c r="B16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="31" t="n">
+      <c r="C16" s="33" t="n">
         <f aca="false">SUM(C11:C15)</f>
         <v>1315174.15352059</v>
       </c>
-      <c r="D16" s="31" t="n">
+      <c r="D16" s="33" t="n">
         <f aca="false">SUM(D11:D15)</f>
         <v>1934607.64755675</v>
       </c>
-      <c r="E16" s="31" t="n">
+      <c r="E16" s="33" t="n">
         <f aca="false">SUM(E11:E15)</f>
         <v>2593479.21796845</v>
       </c>
-      <c r="F16" s="31" t="n">
+      <c r="F16" s="33" t="n">
         <f aca="false">INDEX(C16:E16,1,Annahmen!$C$4)</f>
         <v>1934607.64755675</v>
       </c>
@@ -4794,19 +5015,19 @@
       <c r="B17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="24" t="n">
+      <c r="C17" s="26" t="n">
         <f aca="false">C16/C6</f>
         <v>36.5326153755718</v>
       </c>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="26" t="n">
         <f aca="false">D16/D6</f>
         <v>41.0570383607121</v>
       </c>
-      <c r="E17" s="24" t="n">
+      <c r="E17" s="26" t="n">
         <f aca="false">E16/E6</f>
         <v>45.3286588826086</v>
       </c>
-      <c r="F17" s="24" t="n">
+      <c r="F17" s="26" t="n">
         <f aca="false">INDEX(C17:E17,1,Annahmen!$C$4)</f>
         <v>41.0570383607121</v>
       </c>
@@ -4917,19 +5138,19 @@
       </c>
       <c r="C6" s="7" t="n">
         <f aca="false">Annahmen!$C$32*Annahmen!$C$33</f>
-        <v>1092000</v>
+        <v>1031513.805</v>
       </c>
       <c r="D6" s="7" t="n">
         <f aca="false">Annahmen!$D$32*Annahmen!$D$33</f>
-        <v>1040000</v>
+        <v>982394.1</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">Annahmen!$E$32*Annahmen!$E$33</f>
-        <v>1040000</v>
+        <v>982394.1</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">INDEX(C6:E6,1,Annahmen!$C$4)</f>
-        <v>1040000</v>
+        <v>982394.1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5081,21 +5302,21 @@
         <v>314</v>
       </c>
       <c r="B13" s="3"/>
-      <c r="C13" s="31" t="n">
+      <c r="C13" s="33" t="n">
         <f aca="false">SUM(C4:C12)</f>
-        <v>1723301.75355906</v>
-      </c>
-      <c r="D13" s="31" t="n">
+        <v>1662815.55855906</v>
+      </c>
+      <c r="D13" s="33" t="n">
         <f aca="false">SUM(D4:D12)</f>
-        <v>1752636.11102732</v>
-      </c>
-      <c r="E13" s="31" t="n">
+        <v>1695030.21102732</v>
+      </c>
+      <c r="E13" s="33" t="n">
         <f aca="false">SUM(E4:E12)</f>
-        <v>1859371.49220854</v>
-      </c>
-      <c r="F13" s="31" t="n">
+        <v>1801765.59220854</v>
+      </c>
+      <c r="F13" s="33" t="n">
         <f aca="false">INDEX(C13:E13,1,Annahmen!$C$4)</f>
-        <v>1752636.11102732</v>
+        <v>1695030.21102732</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5103,21 +5324,21 @@
         <v>315</v>
       </c>
       <c r="B14" s="3"/>
-      <c r="C14" s="31" t="n">
+      <c r="C14" s="33" t="n">
         <f aca="false">Umsatz!C16-C13</f>
-        <v>-408127.600038476</v>
-      </c>
-      <c r="D14" s="31" t="n">
+        <v>-347641.405038476</v>
+      </c>
+      <c r="D14" s="33" t="n">
         <f aca="false">Umsatz!D16-D13</f>
-        <v>181971.536529435</v>
-      </c>
-      <c r="E14" s="31" t="n">
+        <v>239577.436529435</v>
+      </c>
+      <c r="E14" s="33" t="n">
         <f aca="false">Umsatz!E16-E13</f>
-        <v>734107.725759908</v>
-      </c>
-      <c r="F14" s="31" t="n">
+        <v>791713.625759908</v>
+      </c>
+      <c r="F14" s="33" t="n">
         <f aca="false">INDEX(C14:E14,1,Annahmen!$C$4)</f>
-        <v>181971.536529435</v>
+        <v>239577.436529435</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5125,19 +5346,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="3"/>
-      <c r="C15" s="31" t="n">
+      <c r="C15" s="33" t="n">
         <f aca="false">MAX(Annahmen!$C$42,Annahmen!$C$41*Umsatz!C16)</f>
         <v>150000</v>
       </c>
-      <c r="D15" s="31" t="n">
+      <c r="D15" s="33" t="n">
         <f aca="false">MAX(Annahmen!$D$42,Annahmen!$D$41*Umsatz!D16)</f>
         <v>193460.764755675</v>
       </c>
-      <c r="E15" s="31" t="n">
+      <c r="E15" s="33" t="n">
         <f aca="false">MAX(Annahmen!$E$42,Annahmen!$E$41*Umsatz!E16)</f>
         <v>259347.921796845</v>
       </c>
-      <c r="F15" s="31" t="n">
+      <c r="F15" s="33" t="n">
         <f aca="false">INDEX(C15:E15,1,Annahmen!$C$4)</f>
         <v>193460.764755675</v>
       </c>
@@ -5147,21 +5368,21 @@
         <v>316</v>
       </c>
       <c r="B16" s="3"/>
-      <c r="C16" s="31" t="n">
+      <c r="C16" s="33" t="n">
         <f aca="false">C14-C15</f>
-        <v>-558127.600038476</v>
-      </c>
-      <c r="D16" s="31" t="n">
+        <v>-497641.405038476</v>
+      </c>
+      <c r="D16" s="33" t="n">
         <f aca="false">D14-D15</f>
-        <v>-11489.2282262407</v>
-      </c>
-      <c r="E16" s="31" t="n">
+        <v>46116.6717737592</v>
+      </c>
+      <c r="E16" s="33" t="n">
         <f aca="false">E14-E15</f>
-        <v>474759.803963063</v>
-      </c>
-      <c r="F16" s="31" t="n">
+        <v>532365.703963063</v>
+      </c>
+      <c r="F16" s="33" t="n">
         <f aca="false">INDEX(C16:E16,1,Annahmen!$C$4)</f>
-        <v>-11489.2282262407</v>
+        <v>46116.6717737592</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5173,19 +5394,19 @@
       </c>
       <c r="C18" s="9" t="n">
         <f aca="false">C16/Umsatz!C16</f>
-        <v>-0.424375432367209</v>
+        <v>-0.378384416775787</v>
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">D16/Umsatz!D16</f>
-        <v>-0.00593878983201096</v>
+        <v>0.0238377387952543</v>
       </c>
       <c r="E18" s="9" t="n">
         <f aca="false">E16/Umsatz!E16</f>
-        <v>0.183059035396843</v>
+        <v>0.205270857878738</v>
       </c>
       <c r="F18" s="9" t="n">
         <f aca="false">INDEX(C18:E18,1,Annahmen!$C$4)</f>
-        <v>-0.00593878983201096</v>
+        <v>0.0238377387952543</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5197,19 +5418,19 @@
       </c>
       <c r="C19" s="9" t="n">
         <f aca="false">C6/Umsatz!C16</f>
-        <v>0.8303082881281</v>
+        <v>0.784317272536678</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">D6/Umsatz!D16</f>
-        <v>0.537576702600878</v>
+        <v>0.507800173973612</v>
       </c>
       <c r="E19" s="9" t="n">
         <f aca="false">E6/Umsatz!E16</f>
-        <v>0.401005719573363</v>
+        <v>0.378793897091467</v>
       </c>
       <c r="F19" s="9" t="n">
         <f aca="false">INDEX(C19:E19,1,Annahmen!$C$4)</f>
-        <v>0.537576702600878</v>
+        <v>0.507800173973612</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5267,19 +5488,19 @@
       <c r="B22" s="3"/>
       <c r="C22" s="7" t="n">
         <f aca="false">C6+C7+C8+C12</f>
-        <v>1437000</v>
+        <v>1376513.805</v>
       </c>
       <c r="D22" s="7" t="n">
         <f aca="false">D6+D7+D8+D12</f>
-        <v>1345000</v>
+        <v>1287394.1</v>
       </c>
       <c r="E22" s="7" t="n">
         <f aca="false">E6+E7+E8+E12</f>
-        <v>1325000</v>
+        <v>1267394.1</v>
       </c>
       <c r="F22" s="7" t="n">
         <f aca="false">INDEX(C22:E22,1,Annahmen!$C$4)</f>
-        <v>1345000</v>
+        <v>1287394.1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5289,19 +5510,19 @@
       <c r="B23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="24" t="n">
+      <c r="C23" s="26" t="n">
         <f aca="false">(Umsatz!C16*(1-Annahmen!$C$41)-C4-C5-C9-C10-C11)/Umsatz!C6</f>
         <v>24.9265273502629</v>
       </c>
-      <c r="D23" s="24" t="n">
+      <c r="D23" s="26" t="n">
         <f aca="false">(Umsatz!D16*(1-Annahmen!$D$41)-D4-D5-D9-D10-D11)/Umsatz!D6</f>
         <v>28.3003134926519</v>
       </c>
-      <c r="E23" s="24" t="n">
+      <c r="E23" s="26" t="n">
         <f aca="false">(Umsatz!E16*(1-Annahmen!$E$41)-E4-E5-E9-E10-E11)/Umsatz!E6</f>
         <v>31.4560832642325</v>
       </c>
-      <c r="F23" s="24" t="n">
+      <c r="F23" s="26" t="n">
         <f aca="false">INDEX(C23:E23,1,Annahmen!$C$4)</f>
         <v>28.3003134926519</v>
       </c>
@@ -5315,19 +5536,19 @@
       </c>
       <c r="C24" s="7" t="n">
         <f aca="false">C22/C23</f>
-        <v>57649.426244079</v>
+        <v>55222.8469556743</v>
       </c>
       <c r="D24" s="7" t="n">
         <f aca="false">D22/D23</f>
-        <v>47525.9752987974</v>
+        <v>45490.4536776339</v>
       </c>
       <c r="E24" s="7" t="n">
         <f aca="false">E22/E23</f>
-        <v>42122.2181054755</v>
+        <v>40290.9061930512</v>
       </c>
       <c r="F24" s="7" t="n">
         <f aca="false">INDEX(C24:E24,1,Annahmen!$C$4)</f>
-        <v>47525.9752987974</v>
+        <v>45490.4536776339</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5339,19 +5560,19 @@
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">C24/Umsatz!C6</f>
-        <v>1.60137295122442</v>
+        <v>1.53396797099095</v>
       </c>
       <c r="D25" s="9" t="n">
         <f aca="false">D24/Umsatz!D6</f>
-        <v>1.00861577459248</v>
+        <v>0.965417098421772</v>
       </c>
       <c r="E25" s="9" t="n">
         <f aca="false">E24/Umsatz!E6</f>
-        <v>0.736209352538242</v>
+        <v>0.704201803601349</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">INDEX(C25:E25,1,Annahmen!$C$4)</f>
-        <v>1.00861577459248</v>
+        <v>0.965417098421772</v>
       </c>
     </row>
   </sheetData>
@@ -5370,6 +5591,649 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:J35"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="52"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="35" t="s">
+        <v>325</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="B4" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="J4" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <f aca="false">Annahmen!$D$8+Annahmen!$D$9</f>
+        <v>351</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <f aca="false">(B4+B5)*B6</f>
+        <v>4563</v>
+      </c>
+      <c r="J7" s="18"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" s="18" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="J10" s="18" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="J11" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <f aca="false">B8*52-B9*B8-(B10+B11)*B8/5</f>
+        <v>1696</v>
+      </c>
+      <c r="J12" s="18" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="B13" s="26" t="n">
+        <f aca="false">B7/B12</f>
+        <v>2.69044811320755</v>
+      </c>
+      <c r="J13" s="18" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="J14" s="18" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J15" s="18" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="B16" s="20" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J16" s="18" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="B17" s="16" t="n">
+        <v>30000</v>
+      </c>
+      <c r="J17" s="18" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="C20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="16" t="n">
+        <v>4300</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <f aca="false">C20*D20*$B$14</f>
+        <v>60200</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <f aca="false">E20*$B$15</f>
+        <v>3612</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <f aca="false">(E20+F20)*$B$16</f>
+        <v>18505.48</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <f aca="false">E20+F20+G20</f>
+        <v>82317.48</v>
+      </c>
+      <c r="I20" s="26" t="n">
+        <f aca="false">C20*$B$12/$B$7</f>
+        <v>0.371685294762218</v>
+      </c>
+      <c r="J20" s="18" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="C21" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="16" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <f aca="false">C21*D21*$B$14</f>
+        <v>44800</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <f aca="false">E21*$B$15</f>
+        <v>2688</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <f aca="false">(E21+F21)*$B$16</f>
+        <v>13771.52</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <f aca="false">E21+F21+G21</f>
+        <v>61259.52</v>
+      </c>
+      <c r="I21" s="26" t="n">
+        <f aca="false">C21*$B$12/$B$7</f>
+        <v>0.371685294762218</v>
+      </c>
+      <c r="J21" s="18" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="C22" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="16" t="n">
+        <v>3100</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <f aca="false">C22*D22*$B$14</f>
+        <v>43400</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <f aca="false">E22*$B$15</f>
+        <v>2604</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <f aca="false">(E22+F22)*$B$16</f>
+        <v>13341.16</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <f aca="false">E22+F22+G22</f>
+        <v>59345.16</v>
+      </c>
+      <c r="I22" s="26" t="n">
+        <f aca="false">C22*$B$12/$B$7</f>
+        <v>0.371685294762218</v>
+      </c>
+      <c r="J22" s="18" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C23" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="16" t="n">
+        <v>2850</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <f aca="false">C23*D23*$B$14</f>
+        <v>39900</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <f aca="false">E23*$B$15</f>
+        <v>2394</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <f aca="false">(E23+F23)*$B$16</f>
+        <v>12265.26</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <f aca="false">E23+F23+G23</f>
+        <v>54559.26</v>
+      </c>
+      <c r="I23" s="26" t="n">
+        <f aca="false">C23*$B$12/$B$7</f>
+        <v>0.371685294762218</v>
+      </c>
+      <c r="J23" s="18" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C24" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="16" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <f aca="false">C24*D24*$B$14</f>
+        <v>140000</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <f aca="false">E24*$B$15</f>
+        <v>8400</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <f aca="false">(E24+F24)*$B$16</f>
+        <v>43036</v>
+      </c>
+      <c r="H24" s="7" t="n">
+        <f aca="false">E24+F24+G24</f>
+        <v>191436</v>
+      </c>
+      <c r="I24" s="26" t="n">
+        <f aca="false">C24*$B$12/$B$7</f>
+        <v>1.48674117904887</v>
+      </c>
+      <c r="J24" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="C25" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" s="16" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <f aca="false">C25*D25*$B$14</f>
+        <v>123200</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <f aca="false">E25*$B$15</f>
+        <v>7392</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <f aca="false">(E25+F25)*$B$16</f>
+        <v>37871.68</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <f aca="false">E25+F25+G25</f>
+        <v>168463.68</v>
+      </c>
+      <c r="I25" s="26" t="n">
+        <f aca="false">C25*$B$12/$B$7</f>
+        <v>1.48674117904887</v>
+      </c>
+      <c r="J25" s="18" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C26" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <f aca="false">C26*D26*$B$14</f>
+        <v>86100</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <f aca="false">E26*$B$15</f>
+        <v>5166</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <f aca="false">(E26+F26)*$B$16</f>
+        <v>26467.14</v>
+      </c>
+      <c r="H26" s="7" t="n">
+        <f aca="false">E26+F26+G26</f>
+        <v>117733.14</v>
+      </c>
+      <c r="I26" s="26" t="n">
+        <f aca="false">C26*$B$12/$B$7</f>
+        <v>1.11505588428665</v>
+      </c>
+      <c r="J26" s="18" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C27" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="16" t="n">
+        <v>2450</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <f aca="false">C27*D27*$B$14</f>
+        <v>68600</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <f aca="false">E27*$B$15</f>
+        <v>4116</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <f aca="false">(E27+F27)*$B$16</f>
+        <v>21087.64</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <f aca="false">E27+F27+G27</f>
+        <v>93803.64</v>
+      </c>
+      <c r="I27" s="26" t="n">
+        <f aca="false">C27*$B$12/$B$7</f>
+        <v>0.743370589524436</v>
+      </c>
+      <c r="J27" s="18" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C28" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="16" t="n">
+        <v>2150</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <f aca="false">C28*D28*$B$14</f>
+        <v>90300</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <f aca="false">E28*$B$15</f>
+        <v>5418</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <f aca="false">(E28+F28)*$B$16</f>
+        <v>27758.22</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <f aca="false">E28+F28+G28</f>
+        <v>123476.22</v>
+      </c>
+      <c r="I28" s="26" t="n">
+        <f aca="false">C28*$B$12/$B$7</f>
+        <v>1.11505588428665</v>
+      </c>
+      <c r="J28" s="18" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="s">
+        <v>382</v>
+      </c>
+      <c r="C29" s="37" t="n">
+        <f aca="false">SUM(C20:C28)</f>
+        <v>20</v>
+      </c>
+      <c r="E29" s="33" t="n">
+        <f aca="false">SUM(E20:E28)</f>
+        <v>696500</v>
+      </c>
+      <c r="F29" s="33" t="n">
+        <f aca="false">SUM(F20:F28)</f>
+        <v>41790</v>
+      </c>
+      <c r="G29" s="33" t="n">
+        <f aca="false">SUM(G20:G28)</f>
+        <v>214104.1</v>
+      </c>
+      <c r="H29" s="33" t="n">
+        <f aca="false">SUM(H20:H28)</f>
+        <v>952394.1</v>
+      </c>
+      <c r="I29" s="38" t="n">
+        <f aca="false">SUM(I20:I28)</f>
+        <v>7.43370589524436</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <f aca="false">B17</f>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="H31" s="34" t="n">
+        <f aca="false">H29+H30</f>
+        <v>982394.1</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <f aca="false">H31/C29</f>
+        <v>49119.705</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <f aca="false">H31/Umsatz!F16</f>
+        <v>0.507800173973612</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18" t="s">
+        <v>387</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:K26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -5379,7 +6243,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>324</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5393,84 +6257,84 @@
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>325</v>
+        <v>389</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>326</v>
+        <v>390</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>327</v>
+        <v>391</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>328</v>
+        <v>392</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>329</v>
+        <v>393</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>330</v>
+        <v>394</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>331</v>
+        <v>395</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>332</v>
+        <v>396</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>333</v>
+        <v>397</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>334</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="B5" s="33" t="str">
+        <v>399</v>
+      </c>
+      <c r="B5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+0,"0")</f>
         <v>2029</v>
       </c>
-      <c r="C5" s="33" t="str">
+      <c r="C5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+1,"0")</f>
         <v>2030</v>
       </c>
-      <c r="D5" s="33" t="str">
+      <c r="D5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+2,"0")</f>
         <v>2031</v>
       </c>
-      <c r="E5" s="33" t="str">
+      <c r="E5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+3,"0")</f>
         <v>2032</v>
       </c>
-      <c r="F5" s="33" t="str">
+      <c r="F5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+4,"0")</f>
         <v>2033</v>
       </c>
-      <c r="G5" s="33" t="str">
+      <c r="G5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+5,"0")</f>
         <v>2034</v>
       </c>
-      <c r="H5" s="33" t="str">
+      <c r="H5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+6,"0")</f>
         <v>2035</v>
       </c>
-      <c r="I5" s="33" t="str">
+      <c r="I5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+7,"0")</f>
         <v>2036</v>
       </c>
-      <c r="J5" s="33" t="str">
+      <c r="J5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+8,"0")</f>
         <v>2037</v>
       </c>
-      <c r="K5" s="33" t="str">
+      <c r="K5" s="39" t="str">
         <f aca="false">TEXT(Annahmen!$F$50+9,"0")</f>
         <v>2038</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>336</v>
+        <v>400</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">Annahmen!$F$51</f>
@@ -5515,90 +6379,90 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="B7" s="24" t="n">
+        <v>401</v>
+      </c>
+      <c r="B7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^0</f>
         <v>1</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^1</f>
         <v>1.025</v>
       </c>
-      <c r="D7" s="24" t="n">
+      <c r="D7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^2</f>
         <v>1.050625</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^3</f>
         <v>1.076890625</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^4</f>
         <v>1.103812890625</v>
       </c>
-      <c r="G7" s="24" t="n">
+      <c r="G7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^5</f>
         <v>1.13140821289062</v>
       </c>
-      <c r="H7" s="24" t="n">
+      <c r="H7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^6</f>
         <v>1.15969341821289</v>
       </c>
-      <c r="I7" s="24" t="n">
+      <c r="I7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^7</f>
         <v>1.18868575366821</v>
       </c>
-      <c r="J7" s="24" t="n">
+      <c r="J7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^8</f>
         <v>1.21840289750992</v>
       </c>
-      <c r="K7" s="24" t="n">
+      <c r="K7" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$53)^9</f>
         <v>1.24886296994767</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="B8" s="24" t="n">
+        <v>402</v>
+      </c>
+      <c r="B8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^0</f>
         <v>1</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^1</f>
         <v>1.03</v>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^2</f>
         <v>1.0609</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^3</f>
         <v>1.092727</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^4</f>
         <v>1.12550881</v>
       </c>
-      <c r="G8" s="24" t="n">
+      <c r="G8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^5</f>
         <v>1.1592740743</v>
       </c>
-      <c r="H8" s="24" t="n">
+      <c r="H8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^6</f>
         <v>1.194052296529</v>
       </c>
-      <c r="I8" s="24" t="n">
+      <c r="I8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^7</f>
         <v>1.22987386542487</v>
       </c>
-      <c r="J8" s="24" t="n">
+      <c r="J8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^8</f>
         <v>1.26677008138762</v>
       </c>
-      <c r="K8" s="24" t="n">
+      <c r="K8" s="26" t="n">
         <f aca="false">(1+Annahmen!$F$54)^9</f>
         <v>1.30477318382925</v>
       </c>
@@ -5652,50 +6516,50 @@
       <c r="A10" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="31" t="n">
+      <c r="B10" s="33" t="n">
         <f aca="false">Umsatz!F16*B6*B7</f>
         <v>1450955.73566756</v>
       </c>
-      <c r="C10" s="31" t="n">
+      <c r="C10" s="33" t="n">
         <f aca="false">Umsatz!F16*C6*C7</f>
         <v>1784675.5548711</v>
       </c>
-      <c r="D10" s="31" t="n">
+      <c r="D10" s="33" t="n">
         <f aca="false">Umsatz!F16*D6*D7</f>
         <v>2032547.15971431</v>
       </c>
-      <c r="E10" s="31" t="n">
+      <c r="E10" s="33" t="n">
         <f aca="false">Umsatz!F16*E6*E7</f>
         <v>2083360.83870717</v>
       </c>
-      <c r="F10" s="31" t="n">
+      <c r="F10" s="33" t="n">
         <f aca="false">Umsatz!F16*F6*F7</f>
         <v>2135444.85967485</v>
       </c>
-      <c r="G10" s="31" t="n">
+      <c r="G10" s="33" t="n">
         <f aca="false">Umsatz!F16*G6*G7</f>
         <v>2188830.98116672</v>
       </c>
-      <c r="H10" s="31" t="n">
+      <c r="H10" s="33" t="n">
         <f aca="false">Umsatz!F16*H6*H7</f>
         <v>2243551.75569589</v>
       </c>
-      <c r="I10" s="31" t="n">
+      <c r="I10" s="33" t="n">
         <f aca="false">Umsatz!F16*I6*I7</f>
         <v>2299640.54958829</v>
       </c>
-      <c r="J10" s="31" t="n">
+      <c r="J10" s="33" t="n">
         <f aca="false">Umsatz!F16*J6*J7</f>
         <v>2357131.56332799</v>
       </c>
-      <c r="K10" s="31" t="n">
+      <c r="K10" s="33" t="n">
         <f aca="false">Umsatz!F16*K6*K7</f>
         <v>2416059.85241119</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>339</v>
+        <v>403</v>
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">(Betriebskosten!F4+Betriebskosten!F5+Betriebskosten!F9+Betriebskosten!F10+Betriebskosten!F11)*B6*B8</f>
@@ -5744,93 +6608,93 @@
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*B8</f>
-        <v>1345000</v>
+        <v>1287394.1</v>
       </c>
       <c r="C12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*C8</f>
-        <v>1385350</v>
+        <v>1326015.923</v>
       </c>
       <c r="D12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*D8</f>
-        <v>1426910.5</v>
+        <v>1365796.40069</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*E8</f>
-        <v>1469717.815</v>
+        <v>1406770.2927107</v>
       </c>
       <c r="F12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*F8</f>
-        <v>1513809.34945</v>
+        <v>1448973.40149202</v>
       </c>
       <c r="G12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*G8</f>
-        <v>1559223.6299335</v>
+        <v>1492442.60353678</v>
       </c>
       <c r="H12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*H8</f>
-        <v>1606000.33883151</v>
+        <v>1537215.88164289</v>
       </c>
       <c r="I12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*I8</f>
-        <v>1654180.34899645</v>
+        <v>1583332.35809217</v>
       </c>
       <c r="J12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*J8</f>
-        <v>1703805.75946634</v>
+        <v>1630832.32883494</v>
       </c>
       <c r="K12" s="7" t="n">
         <f aca="false">Betriebskosten!F22*K8</f>
-        <v>1754919.93225033</v>
+        <v>1679757.29869999</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>340</v>
+        <v>404</v>
       </c>
       <c r="B13" s="7" t="n">
         <f aca="false">B10-B11-B12</f>
-        <v>-199771.347602924</v>
+        <v>-142165.447602924</v>
       </c>
       <c r="C13" s="7" t="n">
         <f aca="false">C10-C11-C12</f>
-        <v>21446.8799487804</v>
+        <v>80780.9569487802</v>
       </c>
       <c r="D13" s="7" t="n">
         <f aca="false">D10-D11-D12</f>
-        <v>173175.509525432</v>
+        <v>234289.608835432</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">E10-E11-E12</f>
-        <v>168208.039012622</v>
+        <v>231155.561301922</v>
       </c>
       <c r="F13" s="7" t="n">
         <f aca="false">F10-F11-F12</f>
-        <v>162837.475989464</v>
+        <v>227673.423947443</v>
       </c>
       <c r="G13" s="7" t="n">
         <f aca="false">G10-G11-G12</f>
-        <v>157045.375970774</v>
+        <v>223826.402367493</v>
       </c>
       <c r="H13" s="7" t="n">
         <f aca="false">H10-H11-H12</f>
-        <v>150812.582344064</v>
+        <v>219597.039532684</v>
       </c>
       <c r="I13" s="7" t="n">
         <f aca="false">I10-I11-I12</f>
-        <v>144119.201035906</v>
+        <v>214967.191940184</v>
       </c>
       <c r="J13" s="7" t="n">
         <f aca="false">J10-J11-J12</f>
-        <v>136944.574319041</v>
+        <v>209918.004950448</v>
       </c>
       <c r="K13" s="7" t="n">
         <f aca="false">K10-K11-K12</f>
-        <v>129267.253731972</v>
+        <v>204429.887282321</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>341</v>
+        <v>405</v>
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">MAX(Annahmen!$F$42*B8,Annahmen!$F$41*B10)</f>
@@ -5877,90 +6741,90 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="31" t="n">
+      <c r="B15" s="33" t="n">
         <f aca="false">B13-B14</f>
-        <v>-349771.347602924</v>
-      </c>
-      <c r="C15" s="31" t="n">
+        <v>-292165.447602924</v>
+      </c>
+      <c r="C15" s="33" t="n">
         <f aca="false">C13-C14</f>
-        <v>-157020.67553833</v>
-      </c>
-      <c r="D15" s="31" t="n">
+        <v>-97686.5985383302</v>
+      </c>
+      <c r="D15" s="33" t="n">
         <f aca="false">D13-D14</f>
-        <v>-30079.2064459998</v>
-      </c>
-      <c r="E15" s="31" t="n">
+        <v>31034.8928640002</v>
+      </c>
+      <c r="E15" s="33" t="n">
         <f aca="false">E13-E14</f>
-        <v>-40128.0448580948</v>
-      </c>
-      <c r="F15" s="31" t="n">
+        <v>22819.4774312051</v>
+      </c>
+      <c r="F15" s="33" t="n">
         <f aca="false">F13-F14</f>
-        <v>-50707.0099780205</v>
-      </c>
-      <c r="G15" s="31" t="n">
+        <v>14128.9379799583</v>
+      </c>
+      <c r="G15" s="33" t="n">
         <f aca="false">G13-G14</f>
-        <v>-61837.7221458978</v>
-      </c>
-      <c r="H15" s="31" t="n">
+        <v>4943.30425082057</v>
+      </c>
+      <c r="H15" s="33" t="n">
         <f aca="false">H13-H14</f>
-        <v>-73542.5932255253</v>
-      </c>
-      <c r="I15" s="31" t="n">
+        <v>-4758.13603690534</v>
+      </c>
+      <c r="I15" s="33" t="n">
         <f aca="false">I13-I14</f>
-        <v>-85844.8539229228</v>
-      </c>
-      <c r="J15" s="31" t="n">
+        <v>-14996.8630186444</v>
+      </c>
+      <c r="J15" s="33" t="n">
         <f aca="false">J13-J14</f>
-        <v>-98768.5820137584</v>
-      </c>
-      <c r="K15" s="31" t="n">
+        <v>-25795.1513823515</v>
+      </c>
+      <c r="K15" s="33" t="n">
         <f aca="false">K13-K14</f>
-        <v>-112338.731509147</v>
+        <v>-37176.097958798</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>342</v>
+        <v>406</v>
       </c>
       <c r="B16" s="7" t="n">
         <f aca="false">B15</f>
-        <v>-349771.347602924</v>
+        <v>-292165.447602924</v>
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">B16+C15</f>
-        <v>-506792.023141254</v>
+        <v>-389852.046141254</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">C16+D15</f>
-        <v>-536871.229587254</v>
+        <v>-358817.153277254</v>
       </c>
       <c r="E16" s="7" t="n">
         <f aca="false">D16+E15</f>
-        <v>-576999.274445349</v>
+        <v>-335997.675846049</v>
       </c>
       <c r="F16" s="7" t="n">
         <f aca="false">E16+F15</f>
-        <v>-627706.284423369</v>
+        <v>-321868.737866091</v>
       </c>
       <c r="G16" s="7" t="n">
         <f aca="false">F16+G15</f>
-        <v>-689544.006569267</v>
+        <v>-316925.43361527</v>
       </c>
       <c r="H16" s="7" t="n">
         <f aca="false">G16+H15</f>
-        <v>-763086.599794792</v>
+        <v>-321683.569652176</v>
       </c>
       <c r="I16" s="7" t="n">
         <f aca="false">H16+I15</f>
-        <v>-848931.453717715</v>
+        <v>-336680.43267082</v>
       </c>
       <c r="J16" s="7" t="n">
         <f aca="false">I16+J15</f>
-        <v>-947700.035731474</v>
+        <v>-362475.584053172</v>
       </c>
       <c r="K16" s="7" t="n">
         <f aca="false">J16+K15</f>
-        <v>-1060038.76724062</v>
+        <v>-399651.68201197</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5970,7 +6834,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>343</v>
+        <v>407</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">B14</f>
@@ -6015,7 +6879,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>344</v>
+        <v>408</v>
       </c>
       <c r="B19" s="7" t="n">
         <f aca="false">-Investition!$F$49*Annahmen!$F$45*B8</f>
@@ -6060,7 +6924,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>345</v>
+        <v>409</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">-Annahmen!$F$46*B8</f>
@@ -6105,52 +6969,52 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>346</v>
-      </c>
-      <c r="B21" s="31" t="n">
+        <v>410</v>
+      </c>
+      <c r="B21" s="33" t="n">
         <f aca="false">SUM(B18:B20)</f>
         <v>70096</v>
       </c>
-      <c r="C21" s="31" t="n">
+      <c r="C21" s="33" t="n">
         <f aca="false">SUM(C18:C20)</f>
         <v>96166.4354871105</v>
       </c>
-      <c r="D21" s="31" t="n">
+      <c r="D21" s="33" t="n">
         <f aca="false">SUM(D18:D20)</f>
         <v>118484.562371431</v>
       </c>
-      <c r="E21" s="31" t="n">
+      <c r="E21" s="33" t="n">
         <f aca="false">SUM(E18:E20)</f>
         <v>121022.825662717</v>
       </c>
-      <c r="F21" s="31" t="n">
+      <c r="F21" s="33" t="n">
         <f aca="false">SUM(F18:F20)</f>
         <v>123611.830013245</v>
       </c>
-      <c r="G21" s="31" t="n">
+      <c r="G21" s="33" t="n">
         <f aca="false">SUM(G18:G20)</f>
         <v>126252.462483805</v>
       </c>
-      <c r="H21" s="31" t="n">
+      <c r="H21" s="33" t="n">
         <f aca="false">SUM(H18:H20)</f>
         <v>128945.620867736</v>
       </c>
-      <c r="I21" s="31" t="n">
+      <c r="I21" s="33" t="n">
         <f aca="false">SUM(I18:I20)</f>
         <v>131692.21361592</v>
       </c>
-      <c r="J21" s="31" t="n">
+      <c r="J21" s="33" t="n">
         <f aca="false">SUM(J18:J20)</f>
         <v>134493.159749603</v>
       </c>
-      <c r="K21" s="31" t="n">
+      <c r="K21" s="33" t="n">
         <f aca="false">SUM(K18:K20)</f>
         <v>137349.388760427</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>347</v>
+        <v>411</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">B21</f>
@@ -6195,52 +7059,52 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>348</v>
+        <v>412</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*B8</f>
-        <v>23712</v>
+        <v>22398.58548</v>
       </c>
       <c r="C23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*C8</f>
-        <v>24423.36</v>
+        <v>23070.5430444</v>
       </c>
       <c r="D23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*D8</f>
-        <v>25156.0608</v>
+        <v>23762.659335732</v>
       </c>
       <c r="E23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*E8</f>
-        <v>25910.742624</v>
+        <v>24475.539115804</v>
       </c>
       <c r="F23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*F8</f>
-        <v>26688.06490272</v>
+        <v>25209.8052892781</v>
       </c>
       <c r="G23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*G8</f>
-        <v>27488.7068498016</v>
+        <v>25966.0994479564</v>
       </c>
       <c r="H23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*H8</f>
-        <v>28313.3680552957</v>
+        <v>26745.0824313951</v>
       </c>
       <c r="I23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*I8</f>
-        <v>29162.7690969545</v>
+        <v>27547.434904337</v>
       </c>
       <c r="J23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*J8</f>
-        <v>30037.6521698632</v>
+        <v>28373.8579514671</v>
       </c>
       <c r="K23" s="7" t="n">
         <f aca="false">Betriebskosten!F6*Annahmen!$F$48*Annahmen!$F$47*K8</f>
-        <v>30938.7817349591</v>
+        <v>29225.0736900111</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>349</v>
+        <v>413</v>
       </c>
       <c r="B25" s="17" t="n">
         <f aca="false">SUM(B21:K21)</f>
@@ -6249,7 +7113,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>350</v>
+        <v>414</v>
       </c>
       <c r="B26" s="9" t="n">
         <f aca="false">B25/Investition!$F$58</f>
@@ -6267,7 +7131,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6287,24 +7151,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>351</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="34" t="s">
-        <v>352</v>
-      </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
+      <c r="A2" s="40" t="s">
+        <v>416</v>
+      </c>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>353</v>
+        <v>417</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">Investition!$F$58</f>
@@ -6313,63 +7177,63 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="D5" s="27" t="n">
+        <v>418</v>
+      </c>
+      <c r="D5" s="29" t="n">
         <v>0.1</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>355</v>
+        <v>419</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="D6" s="27" t="n">
+        <v>420</v>
+      </c>
+      <c r="D6" s="29" t="n">
         <v>0.15</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>357</v>
+        <v>421</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="D7" s="27" t="n">
+        <v>422</v>
+      </c>
+      <c r="D7" s="29" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>359</v>
+        <v>423</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>360</v>
+        <v>424</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>361</v>
+        <v>425</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>362</v>
+        <v>426</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>363</v>
+        <v>427</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>364</v>
+        <v>428</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>365</v>
+        <v>429</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>366</v>
+        <v>430</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>367</v>
+        <v>431</v>
       </c>
       <c r="B10" s="19" t="n">
         <v>5700</v>
@@ -6377,7 +7241,7 @@
       <c r="C10" s="19" t="n">
         <v>75000</v>
       </c>
-      <c r="D10" s="35"/>
+      <c r="D10" s="41"/>
       <c r="E10" s="9" t="n">
         <f aca="false">(1-$D$5-$D$6)*($D$7*B10/$B$17+(1-$D$7)*C10/$C$17)+IF(D10="x",$D$6,0)</f>
         <v>0.184313933729822</v>
@@ -6397,7 +7261,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>368</v>
+        <v>432</v>
       </c>
       <c r="B11" s="19" t="n">
         <v>3500</v>
@@ -6405,7 +7269,7 @@
       <c r="C11" s="19" t="n">
         <v>45000</v>
       </c>
-      <c r="D11" s="35"/>
+      <c r="D11" s="41"/>
       <c r="E11" s="9" t="n">
         <f aca="false">(1-$D$5-$D$6)*($D$7*B11/$B$17+(1-$D$7)*C11/$C$17)+IF(D11="x",$D$6,0)</f>
         <v>0.112457519116398</v>
@@ -6425,7 +7289,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>369</v>
+        <v>433</v>
       </c>
       <c r="B12" s="19" t="n">
         <v>1650</v>
@@ -6433,8 +7297,8 @@
       <c r="C12" s="19" t="n">
         <v>120000</v>
       </c>
-      <c r="D12" s="35" t="s">
-        <v>370</v>
+      <c r="D12" s="41" t="s">
+        <v>434</v>
       </c>
       <c r="E12" s="9" t="n">
         <f aca="false">(1-$D$5-$D$6)*($D$7*B12/$B$17+(1-$D$7)*C12/$C$17)+IF(D12="x",$D$6,0)</f>
@@ -6455,7 +7319,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>371</v>
+        <v>435</v>
       </c>
       <c r="B13" s="19" t="n">
         <v>1600</v>
@@ -6463,7 +7327,7 @@
       <c r="C13" s="19" t="n">
         <v>100000</v>
       </c>
-      <c r="D13" s="35"/>
+      <c r="D13" s="41"/>
       <c r="E13" s="9" t="n">
         <f aca="false">(1-$D$5-$D$6)*($D$7*B13/$B$17+(1-$D$7)*C13/$C$17)+IF(D13="x",$D$6,0)</f>
         <v>0.105564995751912</v>
@@ -6483,7 +7347,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>372</v>
+        <v>436</v>
       </c>
       <c r="B14" s="19" t="n">
         <v>1550</v>
@@ -6491,7 +7355,7 @@
       <c r="C14" s="19" t="n">
         <v>75000</v>
       </c>
-      <c r="D14" s="35"/>
+      <c r="D14" s="41"/>
       <c r="E14" s="9" t="n">
         <f aca="false">(1-$D$5-$D$6)*($D$7*B14/$B$17+(1-$D$7)*C14/$C$17)+IF(D14="x",$D$6,0)</f>
         <v>0.0873513169073917</v>
@@ -6511,7 +7375,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>373</v>
+        <v>437</v>
       </c>
       <c r="B15" s="19" t="n">
         <v>1200</v>
@@ -6519,7 +7383,7 @@
       <c r="C15" s="19" t="n">
         <v>70000</v>
       </c>
-      <c r="D15" s="35"/>
+      <c r="D15" s="41"/>
       <c r="E15" s="9" t="n">
         <f aca="false">(1-$D$5-$D$6)*($D$7*B15/$B$17+(1-$D$7)*C15/$C$17)+IF(D15="x",$D$6,0)</f>
         <v>0.0757646559048428</v>
@@ -6539,7 +7403,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>374</v>
+        <v>438</v>
       </c>
       <c r="B16" s="19" t="n">
         <v>850</v>
@@ -6547,7 +7411,7 @@
       <c r="C16" s="19" t="n">
         <v>65000</v>
       </c>
-      <c r="D16" s="35"/>
+      <c r="D16" s="41"/>
       <c r="E16" s="9" t="n">
         <f aca="false">(1-$D$5-$D$6)*($D$7*B16/$B$17+(1-$D$7)*C16/$C$17)+IF(D16="x",$D$6,0)</f>
         <v>0.064177994902294</v>
@@ -6567,36 +7431,36 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>375</v>
-      </c>
-      <c r="B17" s="31" t="n">
+        <v>439</v>
+      </c>
+      <c r="B17" s="33" t="n">
         <f aca="false">SUM(B10:B16)</f>
         <v>16050</v>
       </c>
-      <c r="C17" s="31" t="n">
+      <c r="C17" s="33" t="n">
         <f aca="false">SUM(C10:C16)</f>
         <v>550000</v>
       </c>
-      <c r="E17" s="36" t="n">
+      <c r="E17" s="42" t="n">
         <f aca="false">SUM(E10:E16)</f>
         <v>0.9</v>
       </c>
-      <c r="F17" s="31" t="n">
+      <c r="F17" s="33" t="n">
         <f aca="false">SUM(F10:F16)</f>
         <v>7701502.32</v>
       </c>
-      <c r="G17" s="31" t="n">
+      <c r="G17" s="33" t="n">
         <f aca="false">SUM(G10:G16)</f>
         <v>118811.449901199</v>
       </c>
-      <c r="H17" s="31" t="n">
+      <c r="H17" s="33" t="n">
         <f aca="false">F17/B17</f>
         <v>479.844381308411</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>376</v>
+        <v>440</v>
       </c>
       <c r="E18" s="9" t="n">
         <f aca="false">D5</f>
@@ -6609,7 +7473,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>377</v>
+        <v>441</v>
       </c>
       <c r="E19" s="21" t="n">
         <f aca="false">E17+E18</f>
@@ -6626,7 +7490,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>378</v>
+        <v>442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>